<commit_message>
Update the Locators For the Payroll And Sales Module
Update The Locators For the Sales Cataloug Price, Customer Items Locators, Sales PriceList Locators, Approval Page Locators And Attendance Leave Locators Then Some Minor Changes In The Customer Schedule Functions
</commit_message>
<xml_diff>
--- a/testdata/CUST SCH.xlsx
+++ b/testdata/CUST SCH.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="16215" windowHeight="5535" firstSheet="10" activeTab="11"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="16215" windowHeight="5535" firstSheet="17" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="SO Domestic PL (S&amp;D)" sheetId="25" r:id="rId1"/>
@@ -118,7 +118,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4575" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4509" uniqueCount="254">
   <si>
     <t>Item</t>
   </si>
@@ -777,15 +777,6 @@
     <t>HK-FG-CS-308129</t>
   </si>
   <si>
-    <t>HK-FG-CS-149487</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-953393</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-771112</t>
-  </si>
-  <si>
     <t>HK-FG-CS-918483</t>
   </si>
   <si>
@@ -834,105 +825,6 @@
     <t>31-06-2025</t>
   </si>
   <si>
-    <t>HK-FG-CS-840591</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-319399</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-837047</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-192648</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-253283</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-242075</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-228634</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-211312</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-276075</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-042663</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-048081</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-223213</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-742646</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-093605</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-213674</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-371956</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-360662</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-278617</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-648285</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-658293</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-119708</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-785748</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-249041</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-169676</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-146419</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-814656</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-061411</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-799778</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-887578</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-688005</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-879304</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-990154</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-096859</t>
-  </si>
-  <si>
     <t>HK-FG-CS-271538</t>
   </si>
   <si>
@@ -942,24 +834,6 @@
     <t>HK-FG-CS-574286</t>
   </si>
   <si>
-    <t>HK-FG-CS-409076</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-314020</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-244549</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-313750</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-147937</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-889381</t>
-  </si>
-  <si>
     <t>HK-FG-CS-148867</t>
   </si>
   <si>
@@ -967,6 +841,45 @@
   </si>
   <si>
     <t>HK-FG-CS-554952</t>
+  </si>
+  <si>
+    <t>31-12-2025</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-899326</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-437494</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-510673</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-068419</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-080085</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-490937</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-766363</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-327877</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-199575</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-632727</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-930064</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-064825</t>
   </si>
 </sst>
 </file>
@@ -4376,10 +4289,10 @@
         <v>214</v>
       </c>
       <c r="AL4" s="135" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="AM4" s="135" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:39">
@@ -4395,14 +4308,14 @@
       <c r="D5" s="27">
         <v>2</v>
       </c>
-      <c r="E5" t="s" s="1">
-        <v>271</v>
+      <c r="E5" s="1" t="s">
+        <v>235</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
-      <c r="G5" t="s" s="1">
-        <v>271</v>
+      <c r="G5" s="1" t="s">
+        <v>235</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -4513,7 +4426,7 @@
         <v>28</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:39">
@@ -4529,14 +4442,14 @@
       <c r="D6" s="27">
         <v>1</v>
       </c>
-      <c r="E6" t="s" s="1">
-        <v>272</v>
+      <c r="E6" s="1" t="s">
+        <v>236</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
-      <c r="G6" t="s" s="1">
-        <v>272</v>
+      <c r="G6" s="1" t="s">
+        <v>236</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -4647,7 +4560,7 @@
         <v>28</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="15">
@@ -4663,14 +4576,14 @@
       <c r="D7" s="27">
         <v>3</v>
       </c>
-      <c r="E7" t="s" s="1">
-        <v>273</v>
+      <c r="E7" s="1" t="s">
+        <v>237</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
-      <c r="G7" t="s" s="1">
-        <v>273</v>
+      <c r="G7" s="1" t="s">
+        <v>237</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -4778,10 +4691,10 @@
         <v>213</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="14.25" customHeight="1">
@@ -5135,10 +5048,10 @@
         <v>214</v>
       </c>
       <c r="AL4" s="135" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="AM4" s="135" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:39">
@@ -5154,14 +5067,14 @@
       <c r="D5" s="27">
         <v>2</v>
       </c>
-      <c r="E5" t="s" s="1">
-        <v>280</v>
+      <c r="E5" s="1" t="s">
+        <v>238</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
-      <c r="G5" t="s" s="1">
-        <v>280</v>
+      <c r="G5" s="1" t="s">
+        <v>238</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -5253,7 +5166,7 @@
         <v>195</v>
       </c>
       <c r="AG5" s="136" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="AH5" s="27" t="s">
         <v>209</v>
@@ -5272,7 +5185,7 @@
         <v>28</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:39">
@@ -5288,14 +5201,14 @@
       <c r="D6" s="27">
         <v>1</v>
       </c>
-      <c r="E6" t="s" s="1">
-        <v>281</v>
+      <c r="E6" s="1" t="s">
+        <v>239</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
-      <c r="G6" t="s" s="1">
-        <v>281</v>
+      <c r="G6" s="1" t="s">
+        <v>239</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -5387,7 +5300,7 @@
         <v>195</v>
       </c>
       <c r="AG6" s="136" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="AH6" s="27" t="s">
         <v>207</v>
@@ -5406,7 +5319,7 @@
         <v>28</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="15">
@@ -5422,14 +5335,14 @@
       <c r="D7" s="27">
         <v>3</v>
       </c>
-      <c r="E7" t="s" s="1">
-        <v>282</v>
+      <c r="E7" s="1" t="s">
+        <v>240</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
-      <c r="G7" t="s" s="1">
-        <v>282</v>
+      <c r="G7" s="1" t="s">
+        <v>240</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -5521,7 +5434,7 @@
         <v>195</v>
       </c>
       <c r="AG7" s="136" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="AH7" s="27" t="s">
         <v>208</v>
@@ -5537,10 +5450,10 @@
         <v>213</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="14.25" customHeight="1">
@@ -5894,10 +5807,10 @@
         <v>214</v>
       </c>
       <c r="AL4" s="135" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="AM4" s="135" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:39">
@@ -6025,13 +5938,13 @@
         <v>212</v>
       </c>
       <c r="AK5" s="27" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="AL5" s="27" t="s">
         <v>28</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:39">
@@ -6159,13 +6072,13 @@
         <v>212</v>
       </c>
       <c r="AK6" s="27" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="AL6" s="27" t="s">
         <v>28</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="15">
@@ -6293,13 +6206,13 @@
         <v>212</v>
       </c>
       <c r="AK7" s="27" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="14.25" customHeight="1">
@@ -6653,10 +6566,10 @@
         <v>214</v>
       </c>
       <c r="AL4" s="135" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="AM4" s="135" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:39">
@@ -6673,13 +6586,13 @@
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -6784,13 +6697,13 @@
         <v>212</v>
       </c>
       <c r="AK5" s="27" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="AL5" s="27" t="s">
         <v>28</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:39">
@@ -6807,13 +6720,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -6918,13 +6831,13 @@
         <v>212</v>
       </c>
       <c r="AK6" s="27" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="AL6" s="27" t="s">
         <v>28</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="15">
@@ -6941,13 +6854,13 @@
         <v>3</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -7052,13 +6965,13 @@
         <v>212</v>
       </c>
       <c r="AK7" s="27" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="14.25" customHeight="1">
@@ -7412,10 +7325,10 @@
         <v>214</v>
       </c>
       <c r="AL4" s="135" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="AM4" s="135" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:39">
@@ -7431,14 +7344,14 @@
       <c r="D5" s="27">
         <v>2</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>234</v>
+      <c r="E5" t="s" s="1">
+        <v>251</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>234</v>
+      <c r="G5" t="s" s="1">
+        <v>251</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -7543,13 +7456,13 @@
         <v>212</v>
       </c>
       <c r="AK5" s="27" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="AL5" s="27" t="s">
         <v>28</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:39">
@@ -7565,14 +7478,14 @@
       <c r="D6" s="27">
         <v>1</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>235</v>
+      <c r="E6" t="s" s="1">
+        <v>252</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>235</v>
+      <c r="G6" t="s" s="1">
+        <v>252</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -7677,13 +7590,13 @@
         <v>212</v>
       </c>
       <c r="AK6" s="27" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="AL6" s="27" t="s">
         <v>28</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="15">
@@ -7699,14 +7612,14 @@
       <c r="D7" s="27">
         <v>3</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>236</v>
+      <c r="E7" t="s" s="1">
+        <v>253</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>236</v>
+      <c r="G7" t="s" s="1">
+        <v>253</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -7811,13 +7724,13 @@
         <v>212</v>
       </c>
       <c r="AK7" s="27" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="14.25" customHeight="1">
@@ -8171,10 +8084,10 @@
         <v>214</v>
       </c>
       <c r="AL4" s="135" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="AM4" s="135" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:39">
@@ -8191,13 +8104,13 @@
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -8302,13 +8215,13 @@
         <v>212</v>
       </c>
       <c r="AK5" s="27" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="AL5" s="27" t="s">
         <v>28</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:39">
@@ -8325,13 +8238,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -8436,13 +8349,13 @@
         <v>212</v>
       </c>
       <c r="AK6" s="27" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="AL6" s="27" t="s">
         <v>28</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="15">
@@ -8459,13 +8372,13 @@
         <v>3</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -8570,13 +8483,13 @@
         <v>212</v>
       </c>
       <c r="AK7" s="27" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="14.25" customHeight="1">
@@ -8930,10 +8843,10 @@
         <v>214</v>
       </c>
       <c r="AL4" s="135" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="AM4" s="135" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:39">
@@ -8950,13 +8863,13 @@
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>216</v>
+        <v>248</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>216</v>
+        <v>248</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -9048,7 +8961,7 @@
         <v>195</v>
       </c>
       <c r="AG5" s="136" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="AH5" s="27" t="s">
         <v>209</v>
@@ -9067,7 +8980,7 @@
         <v>28</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:39">
@@ -9084,13 +8997,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>217</v>
+        <v>249</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>217</v>
+        <v>249</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -9182,7 +9095,7 @@
         <v>195</v>
       </c>
       <c r="AG6" s="136" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="AH6" s="27" t="s">
         <v>207</v>
@@ -9201,7 +9114,7 @@
         <v>28</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="15">
@@ -9218,13 +9131,13 @@
         <v>3</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>218</v>
+        <v>250</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>218</v>
+        <v>250</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -9316,7 +9229,7 @@
         <v>195</v>
       </c>
       <c r="AG7" s="136" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="AH7" s="27" t="s">
         <v>208</v>
@@ -9332,10 +9245,10 @@
         <v>215</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="14.25" customHeight="1">
@@ -9689,10 +9602,10 @@
         <v>214</v>
       </c>
       <c r="AL4" s="135" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="AM4" s="135" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:39">
@@ -9709,13 +9622,13 @@
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -9826,7 +9739,7 @@
         <v>28</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:39">
@@ -9843,13 +9756,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -9960,7 +9873,7 @@
         <v>28</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="15">
@@ -9977,13 +9890,13 @@
         <v>3</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -10091,10 +10004,10 @@
         <v>215</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="14.25" customHeight="1">
@@ -11149,10 +11062,10 @@
         <v>214</v>
       </c>
       <c r="AL4" s="135" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="AM4" s="135" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:39">
@@ -11168,14 +11081,14 @@
       <c r="D5" s="27">
         <v>2</v>
       </c>
-      <c r="E5" t="s" s="1">
-        <v>256</v>
+      <c r="E5" s="1" t="s">
+        <v>242</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
-      <c r="G5" t="s" s="1">
-        <v>256</v>
+      <c r="G5" s="1" t="s">
+        <v>242</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -11267,7 +11180,7 @@
         <v>195</v>
       </c>
       <c r="AG5" s="136" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="AH5" s="27" t="s">
         <v>209</v>
@@ -11286,7 +11199,7 @@
         <v>28</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:39">
@@ -11302,14 +11215,14 @@
       <c r="D6" s="27">
         <v>1</v>
       </c>
-      <c r="E6" t="s" s="1">
-        <v>257</v>
+      <c r="E6" s="1" t="s">
+        <v>243</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
-      <c r="G6" t="s" s="1">
-        <v>257</v>
+      <c r="G6" s="1" t="s">
+        <v>243</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -11401,7 +11314,7 @@
         <v>195</v>
       </c>
       <c r="AG6" s="136" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="AH6" s="27" t="s">
         <v>207</v>
@@ -11420,7 +11333,7 @@
         <v>28</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="15">
@@ -11436,14 +11349,14 @@
       <c r="D7" s="27">
         <v>3</v>
       </c>
-      <c r="E7" t="s" s="1">
-        <v>258</v>
+      <c r="E7" s="1" t="s">
+        <v>244</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
-      <c r="G7" t="s" s="1">
-        <v>258</v>
+      <c r="G7" s="1" t="s">
+        <v>244</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -11535,7 +11448,7 @@
         <v>195</v>
       </c>
       <c r="AG7" s="136" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="AH7" s="27" t="s">
         <v>208</v>
@@ -11551,10 +11464,10 @@
         <v>213</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="14.25" customHeight="1">
@@ -11908,10 +11821,10 @@
         <v>214</v>
       </c>
       <c r="AL4" s="135" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="AM4" s="135" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:39">
@@ -11928,13 +11841,13 @@
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>219</v>
+        <v>245</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>219</v>
+        <v>245</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -12026,7 +11939,7 @@
         <v>195</v>
       </c>
       <c r="AG5" s="136" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="AH5" s="27" t="s">
         <v>209</v>
@@ -12045,7 +11958,7 @@
         <v>28</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:39">
@@ -12062,13 +11975,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>220</v>
+        <v>246</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>220</v>
+        <v>246</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -12160,7 +12073,7 @@
         <v>195</v>
       </c>
       <c r="AG6" s="136" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="AH6" s="27" t="s">
         <v>207</v>
@@ -12179,7 +12092,7 @@
         <v>28</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="15">
@@ -12196,13 +12109,13 @@
         <v>3</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>221</v>
+        <v>247</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>221</v>
+        <v>247</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -12294,7 +12207,7 @@
         <v>195</v>
       </c>
       <c r="AG7" s="136" t="s">
-        <v>196</v>
+        <v>241</v>
       </c>
       <c r="AH7" s="27" t="s">
         <v>208</v>
@@ -12310,10 +12223,10 @@
         <v>213</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
Fixes Of Failed Test Scenarios In SO And CS
Fixes Of Failed Test Scenarios In Sales Order, Sales Order Amendment, Customer Schedule And Customer Schedule Amendment Screens
</commit_message>
<xml_diff>
--- a/testdata/CUST SCH.xlsx
+++ b/testdata/CUST SCH.xlsx
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4616" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4622" uniqueCount="275">
   <si>
     <t>Item</t>
   </si>
@@ -936,6 +936,15 @@
   </si>
   <si>
     <t>HK-FG-CS-390602</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-554367</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-871489</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-000324</t>
   </si>
 </sst>
 </file>
@@ -11768,14 +11777,14 @@
       <c r="D5" s="27">
         <v>2</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>239</v>
+      <c r="E5" t="s" s="1">
+        <v>272</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>239</v>
+      <c r="G5" t="s" s="1">
+        <v>272</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -11902,14 +11911,14 @@
       <c r="D6" s="27">
         <v>1</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>240</v>
+      <c r="E6" t="s" s="1">
+        <v>273</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>240</v>
+      <c r="G6" t="s" s="1">
+        <v>273</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -12036,14 +12045,14 @@
       <c r="D7" s="27">
         <v>2</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>241</v>
+      <c r="E7" t="s" s="1">
+        <v>274</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>241</v>
+      <c r="G7" t="s" s="1">
+        <v>274</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>

</xml_diff>

<commit_message>
Fixes Of Sales Order And Sales Order Amendment Screen Scenarios
Fixes Of Sales Order And Sales Order Amendment Screen Scenarios And Direct GRN Service Type
</commit_message>
<xml_diff>
--- a/testdata/CUST SCH.xlsx
+++ b/testdata/CUST SCH.xlsx
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4622" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4630" uniqueCount="279">
   <si>
     <t>Item</t>
   </si>
@@ -945,6 +945,18 @@
   </si>
   <si>
     <t>HK-FG-CS-000324</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-761867</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-255909</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-302997</t>
+  </si>
+  <si>
+    <t>HK-FG-CS-835657</t>
   </si>
 </sst>
 </file>
@@ -4379,14 +4391,14 @@
       <c r="D5" s="27">
         <v>2</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>236</v>
+      <c r="E5" t="s" s="1">
+        <v>278</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>236</v>
+      <c r="G5" t="s" s="1">
+        <v>278</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -5139,13 +5151,13 @@
         <v>2</v>
       </c>
       <c r="E5" t="s" s="1">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" t="s" s="1">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -5273,13 +5285,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="s" s="1">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" t="s" s="1">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -5407,13 +5419,13 @@
         <v>2</v>
       </c>
       <c r="E7" t="s" s="1">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" t="s" s="1">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>

</xml_diff>

<commit_message>
TestData Fixes In New QA Environment For SOM Module
TestData Fixes for The New QA Environment For The sales Order, Sales order Amendment, Customer Schedule , Customer Schedule Amendment And PriceList screens
</commit_message>
<xml_diff>
--- a/testdata/CUST SCH.xlsx
+++ b/testdata/CUST SCH.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="16215" windowHeight="5535" firstSheet="14" activeTab="15"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="16215" windowHeight="5535" firstSheet="13" activeTab="16"/>
   </bookViews>
   <sheets>
     <sheet name="SO Domestic PL (S&amp;D)" sheetId="25" r:id="rId1"/>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4630" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4580" uniqueCount="266">
   <si>
     <t>Item</t>
   </si>
@@ -821,33 +821,6 @@
     <t>HK-FG-CS-023179</t>
   </si>
   <si>
-    <t>HK-FG-CS-817497</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-962648</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-788680</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-519489</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-251739</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-942619</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-197143</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-642717</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-124335</t>
-  </si>
-  <si>
     <t>HK-FG-CS-888457</t>
   </si>
   <si>
@@ -855,15 +828,6 @@
   </si>
   <si>
     <t>HK-FG-CS-121525</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-919288</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-272582</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-184687</t>
   </si>
   <si>
     <t>HK-FG-CS-554008</t>
@@ -884,79 +848,76 @@
     <t>HK-FG-CS-799277</t>
   </si>
   <si>
-    <t>HK-FG-CS-973206</t>
+    <t>HK-FG-CS-414519</t>
   </si>
   <si>
-    <t>HK-FG-CS-050334</t>
+    <t>HK-FG-CS-481967</t>
   </si>
   <si>
-    <t>HK-FG-CS-953111</t>
+    <t>HK-FG-CS-082348</t>
   </si>
   <si>
-    <t>HK-FG-CS-126273</t>
+    <t>HK-FG-CS-259644</t>
   </si>
   <si>
-    <t>HK-FG-CS-083670</t>
+    <t>HK-FG-CS-567621</t>
   </si>
   <si>
-    <t>HK-FG-CS-381588</t>
+    <t>HK-FG-CS-283131</t>
   </si>
   <si>
-    <t>HK-FG-CS-636448</t>
+    <t>HK-FG-CS-038392</t>
   </si>
   <si>
-    <t>HK-FG-CS-717236</t>
+    <t>HK-FG-CS-221473</t>
   </si>
   <si>
-    <t>HK-FG-CS-738238</t>
+    <t>HK-FG-CS-721997</t>
   </si>
   <si>
-    <t>HK-FG-CS-880182</t>
+    <t>HK-FG-CS-071353</t>
   </si>
   <si>
-    <t>HK-FG-CS-210866</t>
+    <t>HK-FG-CS-521662</t>
   </si>
   <si>
-    <t>HK-FG-CS-320543</t>
+    <t>HK-FG-CS-836044</t>
   </si>
   <si>
-    <t>HK-FG-CS-973619</t>
+    <t>HK-FG-CS-487885</t>
   </si>
   <si>
-    <t>HK-FG-CS-195604</t>
+    <t>HK-FG-CS-551794</t>
   </si>
   <si>
-    <t>HK-FG-CS-312399</t>
+    <t>HK-FG-CS-266318</t>
   </si>
   <si>
-    <t>HK-FG-CS-747866</t>
+    <t>HK-FG-CS-588123</t>
   </si>
   <si>
-    <t>HK-FG-CS-841905</t>
+    <t>HK-FG-CS-663353</t>
   </si>
   <si>
-    <t>HK-FG-CS-390602</t>
+    <t>HK-FG-CS-766248</t>
   </si>
   <si>
-    <t>HK-FG-CS-554367</t>
+    <t>HK-FG-CS-902340</t>
   </si>
   <si>
-    <t>HK-FG-CS-871489</t>
+    <t>HK-FG-CS-887728</t>
   </si>
   <si>
-    <t>HK-FG-CS-000324</t>
+    <t>HK-FG-CS-504226</t>
   </si>
   <si>
-    <t>HK-FG-CS-761867</t>
+    <t>HK-FG-CS-205539</t>
   </si>
   <si>
-    <t>HK-FG-CS-255909</t>
+    <t>HK-FG-CS-810701</t>
   </si>
   <si>
-    <t>HK-FG-CS-302997</t>
-  </si>
-  <si>
-    <t>HK-FG-CS-835657</t>
+    <t>HK-FG-CS-077378</t>
   </si>
 </sst>
 </file>
@@ -4391,14 +4352,14 @@
       <c r="D5" s="27">
         <v>2</v>
       </c>
-      <c r="E5" t="s" s="1">
-        <v>278</v>
+      <c r="E5" s="1" t="s">
+        <v>245</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
-      <c r="G5" t="s" s="1">
-        <v>278</v>
+      <c r="G5" s="1" t="s">
+        <v>245</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -4526,13 +4487,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -4660,13 +4621,13 @@
         <v>2</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -5151,13 +5112,13 @@
         <v>2</v>
       </c>
       <c r="E5" t="s" s="1">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" t="s" s="1">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -5198,11 +5159,11 @@
         <f>(L5-P5)</f>
         <v>11880</v>
       </c>
-      <c r="S5" s="27" t="s">
-        <v>183</v>
+      <c r="S5" s="27">
+        <v>88363222</v>
       </c>
       <c r="T5" s="30">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="U5" s="27">
         <f>IF(OR(D5:D6=1,D5:D6=4),ROUND((R5*T5)/2,2),0)</f>
@@ -5214,7 +5175,7 @@
       </c>
       <c r="W5" s="27">
         <f>IF(D5:D6=2,ROUND(((R5*T5)),2),0)</f>
-        <v>1425.6</v>
+        <v>2138.4</v>
       </c>
       <c r="X5" s="27">
         <f>IF(D5:D6=4,ROUND(((R5*T5)/2),2),0)</f>
@@ -5229,11 +5190,11 @@
       </c>
       <c r="AA5" s="27">
         <f t="shared" ref="AA5" si="2">U5+V5+W5+X5+Z5</f>
-        <v>1425.6</v>
+        <v>2138.4</v>
       </c>
       <c r="AB5" s="27">
         <f t="shared" ref="AB5" si="3">R5+AA5</f>
-        <v>13305.6</v>
+        <v>14018.4</v>
       </c>
       <c r="AC5" s="27">
         <v>120</v>
@@ -5285,13 +5246,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="s" s="1">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" t="s" s="1">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -5332,19 +5293,19 @@
         <f>(L6-P6)</f>
         <v>29400</v>
       </c>
-      <c r="S6" s="27" t="s">
-        <v>183</v>
+      <c r="S6" s="27">
+        <v>88363222</v>
       </c>
       <c r="T6" s="30">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="U6" s="27">
         <f>IF(OR(D6:D7=1,D6:D7=4),ROUND((R6*T6)/2,2),0)</f>
-        <v>1764</v>
+        <v>2646</v>
       </c>
       <c r="V6" s="27">
         <f>IF(D6:D7=1,ROUND(((R6*T6)/2),2),0)</f>
-        <v>1764</v>
+        <v>2646</v>
       </c>
       <c r="W6" s="27">
         <f>IF(D6:D7=2,ROUND(((R6*T6)),2),0)</f>
@@ -5363,11 +5324,11 @@
       </c>
       <c r="AA6" s="27">
         <f t="shared" ref="AA6" si="6">U6+V6+W6+X6+Z6</f>
-        <v>3528</v>
+        <v>5292</v>
       </c>
       <c r="AB6" s="27">
         <f t="shared" ref="AB6" si="7">R6+AA6</f>
-        <v>32928</v>
+        <v>34692</v>
       </c>
       <c r="AC6" s="27">
         <v>120</v>
@@ -5419,13 +5380,13 @@
         <v>2</v>
       </c>
       <c r="E7" t="s" s="1">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" t="s" s="1">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -5466,11 +5427,11 @@
         <f>(L7-P7)</f>
         <v>52380</v>
       </c>
-      <c r="S7" s="27" t="s">
-        <v>183</v>
+      <c r="S7" s="27">
+        <v>88363222</v>
       </c>
       <c r="T7" s="30">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="U7" s="27">
         <f>IF(OR(D7:D8=1,D7:D8=4),ROUND((R7*T7)/2,2),0)</f>
@@ -5482,7 +5443,7 @@
       </c>
       <c r="W7" s="27">
         <f>IF(D7:D8=2,ROUND(((R7*T7)),2),0)</f>
-        <v>6285.6</v>
+        <v>9428.4</v>
       </c>
       <c r="X7" s="27">
         <f>IF(D7:D8=4,ROUND(((R7*T7)/2),2),0)</f>
@@ -5497,7 +5458,7 @@
       </c>
       <c r="AA7" s="27">
         <f t="shared" ref="AA7" si="10">U7+V7+W7+X7+Z7</f>
-        <v>6285.6</v>
+        <v>9428.4</v>
       </c>
       <c r="AB7" s="27">
         <f>R7</f>
@@ -5571,7 +5532,7 @@
       <c r="AA8" s="15"/>
       <c r="AB8" s="79">
         <f>SUM(AB5:AB7)</f>
-        <v>98613.6</v>
+        <v>101090.4</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>40</v>
@@ -5957,8 +5918,8 @@
         <f>(L5-P5)</f>
         <v>11880</v>
       </c>
-      <c r="S5" s="27" t="s">
-        <v>183</v>
+      <c r="S5" s="27">
+        <v>88363222</v>
       </c>
       <c r="T5" s="30">
         <v>0.18</v>
@@ -6091,19 +6052,19 @@
         <f>(L6-P6)</f>
         <v>29400</v>
       </c>
-      <c r="S6" s="27" t="s">
-        <v>183</v>
+      <c r="S6" s="27">
+        <v>88363222</v>
       </c>
       <c r="T6" s="30">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="U6" s="27">
         <f>IF(OR(D6:D7=1,D6:D7=4),ROUND((R6*T6)/2,2),0)</f>
-        <v>1764</v>
+        <v>2646</v>
       </c>
       <c r="V6" s="27">
         <f>IF(D6:D7=1,ROUND(((R6*T6)/2),2),0)</f>
-        <v>1764</v>
+        <v>2646</v>
       </c>
       <c r="W6" s="27">
         <f>IF(D6:D7=2,ROUND(((R6*T6)),2),0)</f>
@@ -6122,11 +6083,11 @@
       </c>
       <c r="AA6" s="27">
         <f t="shared" si="2"/>
-        <v>3528</v>
+        <v>5292</v>
       </c>
       <c r="AB6" s="27">
         <f t="shared" si="3"/>
-        <v>32928</v>
+        <v>34692</v>
       </c>
       <c r="AC6" s="27">
         <v>120</v>
@@ -6225,8 +6186,8 @@
         <f>(L7-P7)</f>
         <v>52380</v>
       </c>
-      <c r="S7" s="27" t="s">
-        <v>183</v>
+      <c r="S7" s="27">
+        <v>88363222</v>
       </c>
       <c r="T7" s="30">
         <v>0.18</v>
@@ -6330,7 +6291,7 @@
       <c r="AA8" s="15"/>
       <c r="AB8" s="79">
         <f>SUM(AB5:AB7)</f>
-        <v>99326.399999999994</v>
+        <v>101090.4</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>40</v>
@@ -6716,8 +6677,8 @@
         <f>(L5-P5)</f>
         <v>21600</v>
       </c>
-      <c r="S5" s="27" t="s">
-        <v>183</v>
+      <c r="S5" s="27">
+        <v>88363222</v>
       </c>
       <c r="T5" s="30">
         <v>0.18</v>
@@ -6850,19 +6811,19 @@
         <f>(L6-P6)</f>
         <v>54000</v>
       </c>
-      <c r="S6" s="27" t="s">
-        <v>183</v>
+      <c r="S6" s="27">
+        <v>88363222</v>
       </c>
       <c r="T6" s="30">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="U6" s="27">
         <f>IF(OR(D6:D7=1,D6:D7=4),ROUND((R6*T6)/2,2),0)</f>
-        <v>3240</v>
+        <v>4860</v>
       </c>
       <c r="V6" s="27">
         <f>IF(D6:D7=1,ROUND(((R6*T6)/2),2),0)</f>
-        <v>3240</v>
+        <v>4860</v>
       </c>
       <c r="W6" s="27">
         <f>IF(D6:D7=2,ROUND(((R6*T6)),2),0)</f>
@@ -6881,11 +6842,11 @@
       </c>
       <c r="AA6" s="27">
         <f t="shared" si="2"/>
-        <v>6480</v>
+        <v>9720</v>
       </c>
       <c r="AB6" s="27">
         <f t="shared" si="3"/>
-        <v>60480</v>
+        <v>63720</v>
       </c>
       <c r="AC6" s="27">
         <v>120</v>
@@ -6984,8 +6945,8 @@
         <f>(L7-P7)</f>
         <v>97200</v>
       </c>
-      <c r="S7" s="27" t="s">
-        <v>183</v>
+      <c r="S7" s="27">
+        <v>88363222</v>
       </c>
       <c r="T7" s="30">
         <v>0.18</v>
@@ -7089,7 +7050,7 @@
       <c r="AA8" s="15"/>
       <c r="AB8" s="79">
         <f>SUM(AB5:AB7)</f>
-        <v>183168</v>
+        <v>186408</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>40</v>
@@ -7428,13 +7389,13 @@
         <v>1</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -7562,13 +7523,13 @@
         <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="F6" s="80">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -8053,13 +8014,13 @@
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -8100,8 +8061,8 @@
         <f>(L5-P5)</f>
         <v>21600</v>
       </c>
-      <c r="S5" s="27" t="s">
-        <v>183</v>
+      <c r="S5" s="27">
+        <v>88363222</v>
       </c>
       <c r="T5" s="30">
         <v>0.18</v>
@@ -8187,13 +8148,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -8234,19 +8195,19 @@
         <f>(L6-P6)</f>
         <v>54000</v>
       </c>
-      <c r="S6" s="27" t="s">
-        <v>183</v>
+      <c r="S6" s="27">
+        <v>88363222</v>
       </c>
       <c r="T6" s="30">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="U6" s="27">
         <f>IF(OR(D6:D7=1,D6:D7=4),ROUND((R6*T6)/2,2),0)</f>
-        <v>3240</v>
+        <v>4860</v>
       </c>
       <c r="V6" s="27">
         <f>IF(D6:D7=1,ROUND(((R6*T6)/2),2),0)</f>
-        <v>3240</v>
+        <v>4860</v>
       </c>
       <c r="W6" s="27">
         <f>IF(D6:D7=2,ROUND(((R6*T6)),2),0)</f>
@@ -8265,11 +8226,11 @@
       </c>
       <c r="AA6" s="27">
         <f t="shared" si="2"/>
-        <v>6480</v>
+        <v>9720</v>
       </c>
       <c r="AB6" s="27">
         <f t="shared" si="3"/>
-        <v>60480</v>
+        <v>63720</v>
       </c>
       <c r="AC6" s="27">
         <v>120</v>
@@ -8321,13 +8282,13 @@
         <v>2</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -8368,8 +8329,8 @@
         <f>(L7-P7)</f>
         <v>97200</v>
       </c>
-      <c r="S7" s="27" t="s">
-        <v>183</v>
+      <c r="S7" s="27">
+        <v>88363222</v>
       </c>
       <c r="T7" s="30">
         <v>0.18</v>
@@ -8473,7 +8434,7 @@
       <c r="AA8" s="15"/>
       <c r="AB8" s="79">
         <f>SUM(AB5:AB7)</f>
-        <v>183168</v>
+        <v>186408</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>40</v>
@@ -8811,14 +8772,14 @@
       <c r="D5" s="27">
         <v>2</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>248</v>
+      <c r="E5" t="s" s="1">
+        <v>257</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>248</v>
+      <c r="G5" t="s" s="1">
+        <v>257</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -8859,8 +8820,8 @@
         <f>(L5-P5)</f>
         <v>23760</v>
       </c>
-      <c r="S5" s="27" t="s">
-        <v>183</v>
+      <c r="S5" s="27">
+        <v>88363222</v>
       </c>
       <c r="T5" s="30">
         <v>0.18</v>
@@ -8945,14 +8906,14 @@
       <c r="D6" s="27">
         <v>1</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>249</v>
+      <c r="E6" t="s" s="1">
+        <v>258</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>249</v>
+      <c r="G6" t="s" s="1">
+        <v>258</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -8993,19 +8954,19 @@
         <f>(L6-P6)</f>
         <v>58800</v>
       </c>
-      <c r="S6" s="27" t="s">
-        <v>183</v>
+      <c r="S6" s="27">
+        <v>88363222</v>
       </c>
       <c r="T6" s="30">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="U6" s="27">
         <f>IF(OR(D6:D7=1,D6:D7=4),ROUND((R6*T6)/2,2),0)</f>
-        <v>3528</v>
+        <v>5292</v>
       </c>
       <c r="V6" s="27">
         <f>IF(D6:D7=1,ROUND(((R6*T6)/2),2),0)</f>
-        <v>3528</v>
+        <v>5292</v>
       </c>
       <c r="W6" s="27">
         <f>IF(D6:D7=2,ROUND(((R6*T6)),2),0)</f>
@@ -9024,11 +8985,11 @@
       </c>
       <c r="AA6" s="27">
         <f t="shared" si="2"/>
-        <v>7056</v>
+        <v>10584</v>
       </c>
       <c r="AB6" s="27">
         <f t="shared" si="3"/>
-        <v>65856</v>
+        <v>69384</v>
       </c>
       <c r="AC6" s="27">
         <v>120</v>
@@ -9079,14 +9040,14 @@
       <c r="D7" s="27">
         <v>2</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>250</v>
+      <c r="E7" t="s" s="1">
+        <v>259</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>250</v>
+      <c r="G7" t="s" s="1">
+        <v>259</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -9127,8 +9088,8 @@
         <f>(L7-P7)</f>
         <v>104760</v>
       </c>
-      <c r="S7" s="27" t="s">
-        <v>183</v>
+      <c r="S7" s="27">
+        <v>88363222</v>
       </c>
       <c r="T7" s="30">
         <v>0.18</v>
@@ -9232,7 +9193,7 @@
       <c r="AA8" s="15"/>
       <c r="AB8" s="79">
         <f>SUM(AB5:AB7)</f>
-        <v>198652.79999999999</v>
+        <v>202180.8</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>40</v>
@@ -9571,13 +9532,13 @@
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -9618,8 +9579,8 @@
         <f>(L5-P5)</f>
         <v>11880</v>
       </c>
-      <c r="S5" s="27" t="s">
-        <v>183</v>
+      <c r="S5" s="27">
+        <v>88363222</v>
       </c>
       <c r="T5" s="30">
         <v>0.18</v>
@@ -9705,13 +9666,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -9752,19 +9713,19 @@
         <f>(L6-P6)</f>
         <v>29400</v>
       </c>
-      <c r="S6" s="27" t="s">
-        <v>183</v>
+      <c r="S6" s="27">
+        <v>88363222</v>
       </c>
       <c r="T6" s="30">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="U6" s="27">
         <f>IF(OR(D6:D7=1,D6:D7=4),ROUND((R6*T6)/2,2),0)</f>
-        <v>1764</v>
+        <v>2646</v>
       </c>
       <c r="V6" s="27">
         <f>IF(D6:D7=1,ROUND(((R6*T6)/2),2),0)</f>
-        <v>1764</v>
+        <v>2646</v>
       </c>
       <c r="W6" s="27">
         <f>IF(D6:D7=2,ROUND(((R6*T6)),2),0)</f>
@@ -9783,11 +9744,11 @@
       </c>
       <c r="AA6" s="27">
         <f t="shared" si="2"/>
-        <v>3528</v>
+        <v>5292</v>
       </c>
       <c r="AB6" s="27">
         <f t="shared" si="3"/>
-        <v>32928</v>
+        <v>34692</v>
       </c>
       <c r="AC6" s="27">
         <v>120</v>
@@ -9839,13 +9800,13 @@
         <v>2</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -9886,8 +9847,8 @@
         <f>(L7-P7)</f>
         <v>52380</v>
       </c>
-      <c r="S7" s="27" t="s">
-        <v>183</v>
+      <c r="S7" s="27">
+        <v>88363222</v>
       </c>
       <c r="T7" s="30">
         <v>0.18</v>
@@ -9991,7 +9952,7 @@
       <c r="AA8" s="15"/>
       <c r="AB8" s="79">
         <f>SUM(AB5:AB7)</f>
-        <v>99326.399999999994</v>
+        <v>101090.4</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>40</v>
@@ -11078,8 +11039,8 @@
         <f>(L5-P5)</f>
         <v>11880</v>
       </c>
-      <c r="S5" s="27" t="s">
-        <v>183</v>
+      <c r="S5" s="27">
+        <v>88363222</v>
       </c>
       <c r="T5" s="30">
         <v>0.18</v>
@@ -11212,19 +11173,19 @@
         <f>(L6-P6)</f>
         <v>29400</v>
       </c>
-      <c r="S6" s="27" t="s">
-        <v>183</v>
+      <c r="S6" s="27">
+        <v>88363222</v>
       </c>
       <c r="T6" s="30">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="U6" s="27">
         <f>IF(OR(D6:D7=1,D6:D7=4),ROUND((R6*T6)/2,2),0)</f>
-        <v>1764</v>
+        <v>2646</v>
       </c>
       <c r="V6" s="27">
         <f>IF(D6:D7=1,ROUND(((R6*T6)/2),2),0)</f>
-        <v>1764</v>
+        <v>2646</v>
       </c>
       <c r="W6" s="27">
         <f>IF(D6:D7=2,ROUND(((R6*T6)),2),0)</f>
@@ -11243,11 +11204,11 @@
       </c>
       <c r="AA6" s="27">
         <f t="shared" si="2"/>
-        <v>3528</v>
+        <v>5292</v>
       </c>
       <c r="AB6" s="27">
         <f t="shared" si="3"/>
-        <v>32928</v>
+        <v>34692</v>
       </c>
       <c r="AC6" s="27">
         <v>120</v>
@@ -11346,8 +11307,8 @@
         <f>(L7-P7)</f>
         <v>52380</v>
       </c>
-      <c r="S7" s="27" t="s">
-        <v>183</v>
+      <c r="S7" s="27">
+        <v>88363222</v>
       </c>
       <c r="T7" s="30">
         <v>0.18</v>
@@ -11451,7 +11412,7 @@
       <c r="AA8" s="15"/>
       <c r="AB8" s="79">
         <f>SUM(AB5:AB7)</f>
-        <v>99326.399999999994</v>
+        <v>101090.4</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>40</v>
@@ -11789,14 +11750,14 @@
       <c r="D5" s="27">
         <v>2</v>
       </c>
-      <c r="E5" t="s" s="1">
-        <v>272</v>
+      <c r="E5" s="1" t="s">
+        <v>248</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
-      <c r="G5" t="s" s="1">
-        <v>272</v>
+      <c r="G5" s="1" t="s">
+        <v>248</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -11837,8 +11798,8 @@
         <f>(L5-P5)</f>
         <v>11880</v>
       </c>
-      <c r="S5" s="27" t="s">
-        <v>183</v>
+      <c r="S5" s="27">
+        <v>88363222</v>
       </c>
       <c r="T5" s="30">
         <v>0.18</v>
@@ -11923,14 +11884,14 @@
       <c r="D6" s="27">
         <v>1</v>
       </c>
-      <c r="E6" t="s" s="1">
-        <v>273</v>
+      <c r="E6" s="1" t="s">
+        <v>249</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
-      <c r="G6" t="s" s="1">
-        <v>273</v>
+      <c r="G6" s="1" t="s">
+        <v>249</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -11971,19 +11932,19 @@
         <f>(L6-P6)</f>
         <v>29400</v>
       </c>
-      <c r="S6" s="27" t="s">
-        <v>183</v>
+      <c r="S6" s="27">
+        <v>88363222</v>
       </c>
       <c r="T6" s="30">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="U6" s="27">
         <f>IF(OR(D6:D7=1,D6:D7=4),ROUND((R6*T6)/2,2),0)</f>
-        <v>1764</v>
+        <v>2646</v>
       </c>
       <c r="V6" s="27">
         <f>IF(D6:D7=1,ROUND(((R6*T6)/2),2),0)</f>
-        <v>1764</v>
+        <v>2646</v>
       </c>
       <c r="W6" s="27">
         <f>IF(D6:D7=2,ROUND(((R6*T6)),2),0)</f>
@@ -12002,11 +11963,11 @@
       </c>
       <c r="AA6" s="27">
         <f t="shared" si="2"/>
-        <v>3528</v>
+        <v>5292</v>
       </c>
       <c r="AB6" s="27">
         <f t="shared" si="3"/>
-        <v>32928</v>
+        <v>34692</v>
       </c>
       <c r="AC6" s="27">
         <v>120</v>
@@ -12057,14 +12018,14 @@
       <c r="D7" s="27">
         <v>2</v>
       </c>
-      <c r="E7" t="s" s="1">
-        <v>274</v>
+      <c r="E7" s="1" t="s">
+        <v>250</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
-      <c r="G7" t="s" s="1">
-        <v>274</v>
+      <c r="G7" s="1" t="s">
+        <v>250</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>
@@ -12105,8 +12066,8 @@
         <f>(L7-P7)</f>
         <v>52380</v>
       </c>
-      <c r="S7" s="27" t="s">
-        <v>183</v>
+      <c r="S7" s="27">
+        <v>88363222</v>
       </c>
       <c r="T7" s="30">
         <v>0.18</v>
@@ -12210,7 +12171,7 @@
       <c r="AA8" s="15"/>
       <c r="AB8" s="79">
         <f>SUM(AB5:AB7)</f>
-        <v>99326.399999999994</v>
+        <v>101090.4</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>40</v>
@@ -12549,13 +12510,13 @@
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="F5" s="27">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="H5" s="27" t="s">
         <v>209</v>
@@ -12683,13 +12644,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="F6" s="27">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="H6" s="27" t="s">
         <v>209</v>
@@ -12817,13 +12778,13 @@
         <v>2</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="F7" s="80">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="H7" s="27" t="s">
         <v>209</v>

</xml_diff>